<commit_message>
M  app/Http/Controllers/App/AppGetSettingsController.php M  "database/seeders/xlsx/dried fruits.xlsx"
</commit_message>
<xml_diff>
--- a/database/seeders/xlsx/dried fruits.xlsx
+++ b/database/seeders/xlsx/dried fruits.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>subcategory_id</t>
   </si>
@@ -81,30 +81,6 @@
   </si>
   <si>
     <t>is_active</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Казахстан</t>
-  </si>
-  <si>
-    <t>Курага</t>
-  </si>
-  <si>
-    <t>Курага — один из самых любимых сухофруктов у тех, кто любит сладкое. Приверженцы здорового образа жизни заменяют ею конфеты и другие сласти, что очень полезно для здоровья.</t>
-  </si>
-  <si>
-    <t>100г.</t>
-  </si>
-  <si>
-    <t>null</t>
-  </si>
-  <si>
-    <t>Инжир</t>
-  </si>
-  <si>
-    <t>Инжир богат калием — его заслуга в снижении высокого давления. Пищевые волокна, которые в избытке содержатся в инжире, улучшают перистальтику кишечника.</t>
   </si>
 </sst>
 </file>
@@ -1039,8 +1015,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="14.7777777777778" customWidth="1"/>
     <col min="2" max="2" width="8.77777777777778" customWidth="1"/>
@@ -1109,118 +1085,6 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I2">
-        <v>215</v>
-      </c>
-      <c r="J2">
-        <v>5.2</v>
-      </c>
-      <c r="K2">
-        <v>0.3</v>
-      </c>
-      <c r="L2">
-        <v>51</v>
-      </c>
-      <c r="M2">
-        <v>320</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>320</v>
-      </c>
-      <c r="P2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q2">
-        <v>1000</v>
-      </c>
-      <c r="R2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I3">
-        <v>257</v>
-      </c>
-      <c r="J3">
-        <v>3.1</v>
-      </c>
-      <c r="K3">
-        <v>0.8</v>
-      </c>
-      <c r="L3">
-        <v>57.9</v>
-      </c>
-      <c r="M3">
-        <v>320</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>320</v>
-      </c>
-      <c r="P3" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q3">
-        <v>1000</v>
-      </c>
-      <c r="R3">
-        <v>1</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>